<commit_message>
Sad - Code works now tho ;/
</commit_message>
<xml_diff>
--- a/USE_THIS_DESIGN_CODE/Input Excel Sheets/Point Performance Requirements/ZW_Snr_Proj_Requirements_Input.xlsx
+++ b/USE_THIS_DESIGN_CODE/Input Excel Sheets/Point Performance Requirements/ZW_Snr_Proj_Requirements_Input.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zackwoj/Documents/MATLAB/26-27/Fall/Aircraft Design/Team06_SeniorProj/USE_THIS_DESIGN_CODE/Input Excel Sheets/Point Performance Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2390B4A6-E194-D340-87C0-1F32B53FE783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02D18B5E-7D0B-A84C-8327-FCC58AB3EA6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" activeTab="1" xr2:uid="{AC12A90C-16A5-0547-A6DB-57534C200D25}"/>
   </bookViews>
   <sheets>
     <sheet name="Templates" sheetId="2" r:id="rId1"/>
-    <sheet name="JB_{V1}" sheetId="10" r:id="rId2"/>
+    <sheet name="JB_V1" sheetId="10" r:id="rId2"/>
     <sheet name="C172" sheetId="3" r:id="rId3"/>
     <sheet name="B747" sheetId="6" r:id="rId4"/>
     <sheet name="TurboTilt" sheetId="8" r:id="rId5"/>

</xml_diff>

<commit_message>
Fixed the point performance guy
</commit_message>
<xml_diff>
--- a/USE_THIS_DESIGN_CODE/Input Excel Sheets/Point Performance Requirements/ZW_Snr_Proj_Requirements_Input.xlsx
+++ b/USE_THIS_DESIGN_CODE/Input Excel Sheets/Point Performance Requirements/ZW_Snr_Proj_Requirements_Input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zackwoj/Documents/MATLAB/26-27/Fall/Aircraft Design/Team06_SeniorProj/USE_THIS_DESIGN_CODE/Input Excel Sheets/Point Performance Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183CC8A0-A5C2-924D-95CC-299F83526B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEE8A906-A9B3-B74A-938F-EBD3FA4668AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" activeTab="1" xr2:uid="{AC12A90C-16A5-0547-A6DB-57534C200D25}"/>
   </bookViews>
@@ -530,7 +530,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -571,12 +571,8 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3185,16 +3181,16 @@
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="10"/>
-      <c r="C3" s="46">
+      <c r="C3" s="42">
         <v>8000</v>
       </c>
-      <c r="D3" s="46">
+      <c r="D3" s="42">
         <v>1.5</v>
       </c>
-      <c r="E3" s="46">
+      <c r="E3" s="42">
         <v>30.414200000000001</v>
       </c>
-      <c r="F3" s="46" t="s">
+      <c r="F3" s="42" t="s">
         <v>20</v>
       </c>
       <c r="K3" s="17"/>
@@ -3249,7 +3245,7 @@
       <c r="F5" s="3">
         <v>1</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="44" t="s">
         <v>32</v>
       </c>
       <c r="H5" s="3">
@@ -3307,7 +3303,7 @@
       <c r="D7" s="2">
         <v>8000</v>
       </c>
-      <c r="E7" s="47" t="s">
+      <c r="E7" s="43" t="s">
         <v>32</v>
       </c>
       <c r="F7" s="36">
@@ -3322,7 +3318,7 @@
       <c r="I7" s="2">
         <v>400</v>
       </c>
-      <c r="J7" s="50" t="s">
+      <c r="J7" s="46" t="s">
         <v>12</v>
       </c>
       <c r="K7" s="17"/>
@@ -3375,9 +3371,9 @@
         <v>0.1</v>
       </c>
       <c r="F9" s="38">
-        <v>1</v>
-      </c>
-      <c r="G9" s="49" t="s">
+        <v>4.4000000000000004</v>
+      </c>
+      <c r="G9" s="45" t="s">
         <v>32</v>
       </c>
       <c r="H9" s="38">
@@ -11615,44 +11611,37 @@
       <c r="B2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="F2" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="43"/>
-      <c r="K2" s="43"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="14"/>
-      <c r="C3" s="43">
+      <c r="C3" s="2">
         <v>1</v>
       </c>
-      <c r="D3" s="43">
+      <c r="D3" s="2">
         <v>5000</v>
       </c>
-      <c r="E3" s="44">
+      <c r="E3" s="36">
         <v>10</v>
       </c>
-      <c r="F3" s="43" t="s">
+      <c r="F3" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="43"/>
-      <c r="H3" s="43"/>
-      <c r="I3" s="43"/>
-      <c r="J3" s="43"/>
-      <c r="K3" s="43"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
@@ -11661,44 +11650,34 @@
       <c r="B4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="40" t="s">
+      <c r="D4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="40" t="s">
+      <c r="E4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="43" t="s">
+      <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="43"/>
-      <c r="H4" s="43"/>
-      <c r="I4" s="43"/>
-      <c r="J4" s="43"/>
-      <c r="K4" s="43"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="5"/>
       <c r="B5" s="14"/>
-      <c r="C5" s="43">
+      <c r="C5" s="2">
         <v>0</v>
       </c>
-      <c r="D5" s="43">
+      <c r="D5" s="2">
         <v>2</v>
       </c>
-      <c r="E5" s="43">
+      <c r="E5" s="2">
         <v>160</v>
       </c>
-      <c r="F5" s="43" t="s">
+      <c r="F5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="43"/>
-      <c r="H5" s="43"/>
-      <c r="I5" s="43"/>
-      <c r="J5" s="43"/>
-      <c r="K5" s="43"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
@@ -11707,62 +11686,62 @@
       <c r="B6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="40" t="s">
+      <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="40" t="s">
+      <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="40" t="s">
+      <c r="E6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F6" s="40" t="s">
+      <c r="F6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="40" t="s">
+      <c r="G6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="40" t="s">
+      <c r="H6" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I6" s="40" t="s">
+      <c r="I6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J6" s="40" t="s">
+      <c r="J6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="43" t="s">
+      <c r="K6" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="5"/>
       <c r="B7" s="14"/>
-      <c r="C7" s="43">
+      <c r="C7" s="2">
         <v>0.85199999999999998</v>
       </c>
-      <c r="D7" s="43">
+      <c r="D7" s="2">
         <v>22500</v>
       </c>
-      <c r="E7" s="43">
+      <c r="E7" s="2">
         <v>0.3</v>
       </c>
-      <c r="F7" s="43">
+      <c r="F7" s="2">
         <v>1</v>
       </c>
-      <c r="G7" s="43" t="s">
+      <c r="G7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="43">
+      <c r="H7" s="2">
         <v>0</v>
       </c>
-      <c r="I7" s="43">
+      <c r="I7" s="2">
         <v>0</v>
       </c>
-      <c r="J7" s="43">
+      <c r="J7" s="2">
         <v>0</v>
       </c>
-      <c r="K7" s="43" t="s">
+      <c r="K7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
@@ -11773,62 +11752,62 @@
       <c r="B8" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C8" s="40" t="s">
+      <c r="C8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="40" t="s">
+      <c r="D8" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E8" s="40" t="s">
+      <c r="E8" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F8" s="40" t="s">
+      <c r="F8" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G8" s="40" t="s">
+      <c r="G8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H8" s="40" t="s">
+      <c r="H8" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I8" s="40" t="s">
+      <c r="I8" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J8" s="40" t="s">
+      <c r="J8" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="K8" s="40" t="s">
+      <c r="K8" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="5"/>
       <c r="B9" s="14"/>
-      <c r="C9" s="43">
+      <c r="C9" s="2">
         <v>0.85199999999999998</v>
       </c>
-      <c r="D9" s="43">
+      <c r="D9" s="2">
         <v>20000</v>
       </c>
-      <c r="E9" s="43">
+      <c r="E9" s="2">
         <v>0.3</v>
       </c>
-      <c r="F9" s="43">
+      <c r="F9" s="2">
         <v>1</v>
       </c>
-      <c r="G9" s="43" t="s">
+      <c r="G9" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H9" s="43">
+      <c r="H9" s="2">
         <v>1.67</v>
       </c>
-      <c r="I9" s="43">
+      <c r="I9" s="2">
         <v>0</v>
       </c>
-      <c r="J9" s="43">
+      <c r="J9" s="2">
         <v>0</v>
       </c>
-      <c r="K9" s="43" t="s">
+      <c r="K9" s="2" t="s">
         <v>28</v>
       </c>
     </row>
@@ -11839,62 +11818,62 @@
       <c r="B10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="40" t="s">
+      <c r="C10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D10" s="40" t="s">
+      <c r="D10" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E10" s="40" t="s">
+      <c r="E10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="F10" s="40" t="s">
+      <c r="F10" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G10" s="40" t="s">
+      <c r="G10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="40" t="s">
+      <c r="H10" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="I10" s="40" t="s">
+      <c r="I10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="J10" s="40" t="s">
+      <c r="J10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="K10" s="40" t="s">
+      <c r="K10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="5"/>
       <c r="B11" s="14"/>
-      <c r="C11" s="43">
+      <c r="C11" s="2">
         <v>0.85199999999999998</v>
       </c>
-      <c r="D11" s="43">
+      <c r="D11" s="2">
         <v>5000</v>
       </c>
-      <c r="E11" s="43">
+      <c r="E11" s="2">
         <v>0.3</v>
       </c>
-      <c r="F11" s="43">
+      <c r="F11" s="2">
         <v>1.5</v>
       </c>
-      <c r="G11" s="43" t="s">
+      <c r="G11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="43">
+      <c r="H11" s="2">
         <v>0</v>
       </c>
-      <c r="I11" s="43">
+      <c r="I11" s="2">
         <v>0</v>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="2">
         <v>0</v>
       </c>
-      <c r="K11" s="43" t="s">
+      <c r="K11" s="2" t="s">
         <v>29</v>
       </c>
     </row>
@@ -11905,103 +11884,94 @@
       <c r="B12" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="45" t="s">
+      <c r="C12" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="40" t="s">
+      <c r="D12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E12" s="45" t="s">
+      <c r="E12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="F12" s="45" t="s">
+      <c r="F12" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="G12" s="45" t="s">
+      <c r="G12" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="45" t="s">
+      <c r="H12" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="I12" s="45" t="s">
+      <c r="I12" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="J12" s="45" t="s">
+      <c r="J12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="K12" s="45" t="s">
+      <c r="K12" s="10" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="5"/>
       <c r="B13" s="14"/>
-      <c r="C13" s="43">
+      <c r="C13" s="2">
         <v>0.85199999999999998</v>
       </c>
-      <c r="D13" s="43">
+      <c r="D13" s="2">
         <v>15000</v>
       </c>
-      <c r="E13" s="43">
+      <c r="E13" s="2">
         <v>0.4</v>
       </c>
-      <c r="F13" s="43">
+      <c r="F13" s="2">
         <v>1</v>
       </c>
-      <c r="G13" s="43" t="s">
+      <c r="G13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="43">
+      <c r="H13" s="2">
         <v>0</v>
       </c>
-      <c r="I13" s="43">
+      <c r="I13" s="2">
         <v>0</v>
       </c>
-      <c r="J13" s="43">
+      <c r="J13" s="2">
         <v>0</v>
       </c>
-      <c r="K13" s="43" t="s">
+      <c r="K13" s="2" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="5"/>
       <c r="B14" s="10"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="40"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
-      <c r="G14" s="45"/>
-      <c r="H14" s="45"/>
-      <c r="I14" s="45"/>
-      <c r="J14" s="45"/>
-      <c r="K14" s="45"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="5"/>
       <c r="B15" s="14"/>
-      <c r="C15" s="43"/>
-      <c r="D15" s="43"/>
-      <c r="E15" s="43"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="43"/>
-      <c r="H15" s="43"/>
-      <c r="I15" s="43"/>
-      <c r="J15" s="43"/>
-      <c r="K15" s="43"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="5"/>
       <c r="B16" s="3"/>
       <c r="C16" s="39"/>
-      <c r="D16" s="40"/>
+      <c r="D16" s="1"/>
       <c r="E16" s="39"/>
       <c r="F16" s="39"/>
       <c r="G16" s="39"/>
       <c r="H16" s="39"/>
-      <c r="I16" s="41"/>
+      <c r="I16" s="40"/>
       <c r="J16" s="39"/>
-      <c r="K16" s="42"/>
+      <c r="K16" s="41"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="5"/>

</xml_diff>